<commit_message>
Completed all 6 tests for the SavingsAccount class and ran them successfully
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_investment_account.xlsx
+++ b/tests/A02_pixell_test_plan_investment_account.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ab840a8a6702860f/Documentos/RRC_Term2/intermediate_software_development/project/isd_project/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="13_ncr:1_{9D6AEFC8-F3D7-467B-9A12-00596A3BA98C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D67D001C-04FE-41D4-8228-A703B7A7590E}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="13_ncr:1_{9D6AEFC8-F3D7-467B-9A12-00596A3BA98C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9D8EF4C-5615-412E-A54C-566C29ECF265}"/>
   <bookViews>
     <workbookView xWindow="-28905" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="32">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -281,6 +281,12 @@
   </si>
   <si>
     <t>InvestmentAccount(1234, 4567, 10000, (2015-9-14), 3.0)</t>
+  </si>
+  <si>
+    <t>Account Number: 1234 Balance: $10,000.00 Date Created:  2024-11-14 Management Fee: Waived Account Type: Investment</t>
+  </si>
+  <si>
+    <t>Account Number: 1234 Balance: $10,000.00 Date Created:  2020-11-14 Management Fee: $3.00 Account Type: Investment</t>
   </si>
 </sst>
 </file>
@@ -1351,7 +1357,7 @@
         <v>23</v>
       </c>
       <c r="G11" s="13">
-        <v>3.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="74.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1370,7 +1376,9 @@
       <c r="F12" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G12" s="13"/>
+      <c r="G12" s="13" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="13" spans="2:7" ht="67.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="11">
@@ -1388,7 +1396,9 @@
       <c r="F13" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G13" s="13"/>
+      <c r="G13" s="13" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="14" spans="2:7" ht="31.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="11">

</xml_diff>

<commit_message>
Updated README file including the Polymorphism section
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_investment_account.xlsx
+++ b/tests/A02_pixell_test_plan_investment_account.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="54" documentId="13_ncr:1_{9D6AEFC8-F3D7-467B-9A12-00596A3BA98C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9D8EF4C-5615-412E-A54C-566C29ECF265}"/>
   <bookViews>
-    <workbookView xWindow="-28905" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1608,9 +1608,10 @@
     <mergeCell ref="B34:G34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>